<commit_message>
Update all amounts to 2026 price levels (x3-4 from 2020 estimates)
- CapEx: ~2.27-3.65M UAH (was 0.58-0.99M), added rent deposit line
- OpEx: ~325-449K UAH/month, breakeven revenue ~0.8-1.1M UAH/month
- Loan scenario: 2.4M UAH, PMT ~53.4K/month, grace period recommended
- Added liquidity reserve recommendation (3 months OpEx)
- Synced figures across XLSX and MD files
</commit_message>
<xml_diff>
--- a/Відкриття_фізичного_магазину.xlsx
+++ b/Відкриття_фізичного_магазину.xlsx
@@ -57,11 +57,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <i val="1"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,14 +141,20 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -528,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -538,7 +544,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>План відкриття фізичного магазину footballshop.com.ua — повна версія</t>
+          <t>План відкриття фізичного магазину footballshop.com.ua — повна версія (ціни 2026)</t>
         </is>
       </c>
     </row>
@@ -574,7 +580,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>5 юридичних конструкцій: суть, механізм, переваги, недоліки, коли доцільно</t>
+          <t>5 юридичних конструкцій: суть, механізм, переваги, недоліки, коли доцільна</t>
         </is>
       </c>
     </row>
@@ -610,7 +616,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Діапазони витрат (мін/макс), беззбитковість, живі формули</t>
+          <t>Діапазони витрат (мін/макс) у цінах 2026, беззбитковість, живі формули</t>
         </is>
       </c>
     </row>
@@ -669,33 +675,41 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>• Суми актуалізовано до цін 2026 року (попередні оцінки 2020 р. збільшено у ~3–4 рази за рішенням власника: інфляція, девальвація, зростання оренди й зарплат).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
           <t>• Усі суми — прогнозні; уточнити під конкретну локацію та орендні ставки.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>• Податкові ставки (станом на 2026) підтвердити з податковим консультантом — норми воєнного часу змінюються.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>• КРИТИЧНО: з 06.01.2026 ПЗ 1С/BAS заборонено в Україні (рішення Держспецзв'язку, штрафи до 2% річного обороту). Bitrix і МойСклад — російського походження. Не використовувати.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="5">
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -949,37 +963,37 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Р6</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Фінансовий</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Девальвація гривні → зростання закупівельних цін (імпорт)</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Висока</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>Високий</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>Критичний</t>
         </is>
       </c>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>Валютне ціноутворення (швидкий перегляд цін); частина запасу — передоплачена; маржинальний буфер</t>
         </is>
@@ -1023,39 +1037,39 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Р8</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Фінансовий</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>Касові розриви на старті (сезонність, повільний розгін)</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Касові розриви на старті (сезонність, повільний розгін; перші 6 міс. — операційний мінус)</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Висока</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Високий</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>Критичний</t>
         </is>
       </c>
-      <c r="G11" s="20" t="inlineStr">
-        <is>
-          <t>Grace period по позиці 6 міс.; резерв ліквідності; контроль cash-flow щотижня</t>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>Grace period по позиці 6–12 міс.; резерв ліквідності ~1,0–1,3 млн грн (3 міс. OpEx); контроль cash-flow щотижня</t>
         </is>
       </c>
     </row>
@@ -1171,37 +1185,37 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Р12</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>Форс-мажор</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Воєнні ризики: пошкодження майна, перебої електропостачання, релокація</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Середня</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="22" t="inlineStr">
         <is>
           <t>Критичний</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>Критичний</t>
         </is>
       </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>Комерційне страхування (пожежа, майно); генератор/EcoFlow для каси; форс-мажорні пункти в усіх договорах; план Б щодо локації</t>
         </is>
@@ -1317,7 +1331,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Закласти в собівартість тарифи доставки (~70–120 грн залежно від ваги, тарифи 2026 уточнити) і пакувальні матеріали</t>
+          <t>Закласти в собівартість тарифи доставки (~80–150 грн залежно від ваги, тарифи 2026 уточнити) і пакувальні матеріали</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1740,7 +1754,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Інвестор зобов'язується надати фінансування в розмірі X грн, що використовується виключно на відкриття і запуск магазину: оренда, ремонт, обладнання, початковий товарний запас, маркетинг запуску.</t>
+          <t>Інвестор зобов'язується надати фінансування в розмірі X грн (орієнтовно 2,4–3,7 млн грн за фінмоделлю), що використовується виключно на відкриття і запуск магазину: оренда, ремонт, обладнання, початковий товарний запас, маркетинг запуску.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1956,7 +1970,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Якщо обороти перевищать поріг обов'язкової реєстрації платником ПДВ (1 млн грн за 12 міс.) — реєстрація обов'язкова. Закупівлі з ПДВ дають податковий кредит.</t>
+          <t>Якщо обороти перевищать поріг обов'язкової реєстрації платником ПДВ (1 млн грн за 12 міс.) — реєстрація обов'язкова. За прогнозної виручки ~10–13 млн грн/рік нове ТОВ стане платником ПДВ практично одразу. Закупівлі з ПДВ дають податковий кредит.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2098,20 +2112,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Фінансова модель: магазин ~40–50 м² (діапазони мін–макс, живі формули)</t>
+          <t>Фінансова модель: магазин ~40–50 м², ціни 2026 (×3–4 від оцінок 2020), живі формули</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2147,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>База розрахунку (мін)</t>
+          <t>Було (оцінка 2020), грн</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2160,12 +2174,16 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>150000</v>
+        <v>500000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D5" s="4" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>150–300 тис.</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Залежить від стану приміщення</t>
@@ -2179,12 +2197,16 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>300000</v>
+        <v>1000000</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>400000</v>
-      </c>
-      <c r="D6" s="4" t="n"/>
+        <v>1400000</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>300–400 тис.</t>
+        </is>
+      </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Глибина асортименту за брендами</t>
@@ -2198,12 +2220,16 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>50000</v>
+        <v>150000</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D7" s="4" t="n"/>
+        <v>200000</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>50 тис.</t>
+        </is>
+      </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Плюс банківський POS-термінал (від банку)</t>
@@ -2217,12 +2243,16 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>25000</v>
+        <v>80000</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>40000</v>
-      </c>
-      <c r="D8" s="4" t="n"/>
+        <v>140000</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>25–40 тис.</t>
+        </is>
+      </c>
       <c r="E8" s="4" t="n"/>
     </row>
     <row r="9">
@@ -2232,12 +2262,16 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>55000</v>
-      </c>
-      <c r="D9" s="4" t="n"/>
+        <v>190000</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>30–55 тис.</t>
+        </is>
+      </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Юрист + реєстраційні платежі</t>
@@ -2251,12 +2285,16 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>60000</v>
+        <v>200000</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90000</v>
-      </c>
-      <c r="D10" s="4" t="n"/>
+        <v>320000</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>60–90 тис.</t>
+        </is>
+      </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Впровадження + інтеграція API</t>
@@ -2266,269 +2304,349 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Завдаток за оренду (2 міс.)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>140000</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>220000</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Повертається або зараховується</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Рекламна кампанія до запуску</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
-        <v>30000</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="B12" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>30–50 тис.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>SMM + локальна реклама + відкриття</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>РАЗОМ CapEx</t>
         </is>
       </c>
-      <c r="B12" s="10">
-        <f>SUM(B5:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="10">
-        <f>SUM(C5:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Орієнтир: ~645–985 тис. грн</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B13" s="10">
+        <f>SUM(B5:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="10">
+        <f>SUM(C5:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Орієнтир: ~2,3–3,7 млн грн</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>+ Рекомендований резерв ліквідності (3 міс. OpEx)</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>3*B23</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>3*C23</f>
+        <v/>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Подушка на касові розриви першого року — НЕ входить у суму CapEx вище</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>OpEx (щомісячні витрати)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Оренда (40–60 м²)</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>30000</v>
-      </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>ТЦ або пішохідна вулиця</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Зарплати: 2 співробітники по ~25 тис. «білої»</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Менеджер + касир</t>
-        </is>
-      </c>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Податки на ФОП (ЄСВ + ПДФО + ВЗ)</t>
+          <t>Оренда (40–60 м², Київ)</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>12000</v>
+        <v>70000</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D16" s="4" t="n"/>
+        <v>110000</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>20–30 тис.</t>
+        </is>
+      </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>~22% ЄСВ + 18% ПДФО + 5% ВЗ</t>
+          <t>ТЦ або пішохідна вулиця</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Комунальні + інтернет</t>
+          <t>Зарплати: 2 співробітники («біла»)</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
+        <v>180000</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>50 тис.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Менеджер + касир, по ~75–90 тис.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Маркетинг / просування</t>
+          <t>Податки на ФОП (ЄСВ 22% тощо)</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>10000</v>
+        <v>33000</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D18" s="4" t="n"/>
+        <v>40000</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>12–15 тис.</t>
+        </is>
+      </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Постійне локальне просування</t>
+          <t>Нараховується на фонд оплати праці</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Інші витрати (упаковка, господарські)</t>
+          <t>Комунальні + інтернет</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D19" s="4" t="n"/>
+        <v>25000</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>5–8 тис.</t>
+        </is>
+      </c>
       <c r="E19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Маркетинг / просування</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>10–15 тис.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Постійне локальне просування</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Інші витрати (упаковка, господарські)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>5–10 тис.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
           <t>Підписки ПЗ (ERP/CRM, ПРРО, POS)</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C20" s="9" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="B22" s="9" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>2–4 тис.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Checkbox + CRM + POS</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>РАЗОМ OpEx / міс.</t>
         </is>
       </c>
-      <c r="B21" s="10">
-        <f>SUM(B14:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="10">
-        <f>SUM(C14:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Орієнтир: ~104–132 тис. грн/міс.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="B23" s="10">
+        <f>SUM(B16:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="10">
+        <f>SUM(C16:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Орієнтир: ~325–449 тис. грн/міс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Беззбитковість</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Середня націнка (маржа у % виручки)</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Параметр — можна змінювати</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Потрібна виручка / міс. (мін. сценарій)</t>
-        </is>
-      </c>
-      <c r="B24" s="10">
-        <f>B21/B23</f>
-        <v/>
-      </c>
-      <c r="C24" s="10">
-        <f>C21/C23</f>
-        <v/>
-      </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>OpEx ÷ маржа</t>
-        </is>
-      </c>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Потрібна виручка / рік</t>
-        </is>
-      </c>
-      <c r="B25" s="9">
-        <f>B24*12</f>
-        <v/>
-      </c>
-      <c r="C25" s="9">
-        <f>C24*12</f>
-        <v/>
+          <t>Середня націнка (маржа у % виручки)</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>0.4</v>
       </c>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>~3,1–4,0 млн грн/рік</t>
+          <t>Параметр — можна змінювати</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Потрібна виручка / міс.</t>
+        </is>
+      </c>
+      <c r="B26" s="10">
+        <f>B23/B26</f>
+        <v/>
+      </c>
+      <c r="C26" s="10">
+        <f>C23/C26</f>
+        <v/>
+      </c>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>OpEx ÷ маржа ≈ 0,8–1,1 млн грн/міс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Потрібна виручка / рік</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>B27*12</f>
+        <v/>
+      </c>
+      <c r="C27" s="9">
+        <f>C27*12</f>
+        <v/>
+      </c>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>≈ 9,8–13,5 млн грн/рік</t>
         </is>
       </c>
     </row>
@@ -2546,29 +2664,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Помісячний прогноз першого року роботи (P&amp;L), грн — листопад 2026 – жовтень 2027</t>
+          <t>Помісячний прогноз першого року роботи (P&amp;L), грн — листопад 2026 – жовтень 2027, ціни 2026</t>
         </is>
       </c>
     </row>
@@ -2650,43 +2768,43 @@
           <t>Виручка</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="C4" s="12" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>160000</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>260000</v>
-      </c>
-      <c r="H4" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>300000</v>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>290000</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>300000</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>310000</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>320000</v>
-      </c>
-      <c r="N4" s="12">
+      <c r="B4" s="14" t="n">
+        <v>420000</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>700000</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>525000</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>560000</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>770000</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>910000</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>980000</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>1015000</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>1120000</v>
+      </c>
+      <c r="N4" s="14">
         <f>SUM(B4:M4)</f>
         <v/>
       </c>
@@ -2697,21 +2815,21 @@
           <t>Маржа (параметр)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
-      <c r="I5" s="14" t="n"/>
-      <c r="J5" s="14" t="n"/>
-      <c r="K5" s="14" t="n"/>
-      <c r="L5" s="14" t="n"/>
-      <c r="M5" s="14" t="n"/>
-      <c r="N5" s="14" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
+      <c r="M5" s="16" t="n"/>
+      <c r="N5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2719,55 +2837,55 @@
           <t>Валовий прибуток (виручка × маржа)</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="14">
         <f>B4*$B$5</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="14">
         <f>C4*$B$5</f>
         <v/>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="14">
         <f>D4*$B$5</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="14">
         <f>E4*$B$5</f>
         <v/>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="14">
         <f>F4*$B$5</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="14">
         <f>G4*$B$5</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="14">
         <f>H4*$B$5</f>
         <v/>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="14">
         <f>I4*$B$5</f>
         <v/>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="14">
         <f>J4*$B$5</f>
         <v/>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="14">
         <f>K4*$B$5</f>
         <v/>
       </c>
-      <c r="L6" s="12">
+      <c r="L6" s="14">
         <f>L4*$B$5</f>
         <v/>
       </c>
-      <c r="M6" s="12">
+      <c r="M6" s="14">
         <f>M4*$B$5</f>
         <v/>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="14">
         <f>SUM(B6:M6)</f>
         <v/>
       </c>
@@ -2778,43 +2896,43 @@
           <t>OpEx (постійні витрати)</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="K7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="L7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="M7" s="12" t="n">
-        <v>110000</v>
-      </c>
-      <c r="N7" s="12">
+      <c r="B7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v>380000</v>
+      </c>
+      <c r="N7" s="14">
         <f>SUM(B7:M7)</f>
         <v/>
       </c>
@@ -2825,55 +2943,55 @@
           <t>Операційний прибуток</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="14">
         <f>B6-B7</f>
         <v/>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="14">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <f>D6-D7</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="14">
         <f>E6-E7</f>
         <v/>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="14">
         <f>F6-F7</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="14">
         <f>G6-G7</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="14">
         <f>H6-H7</f>
         <v/>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="14">
         <f>I6-I7</f>
         <v/>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="14">
         <f>J6-J7</f>
         <v/>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="14">
         <f>K6-K7</f>
         <v/>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="14">
         <f>L6-L7</f>
         <v/>
       </c>
-      <c r="M8" s="12">
+      <c r="M8" s="14">
         <f>M6-M7</f>
         <v/>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="14">
         <f>SUM(B8:M8)</f>
         <v/>
       </c>
@@ -2884,55 +3002,55 @@
           <t>Наростаючий підсумок (cash від операцій)</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="14">
         <f>B8</f>
         <v/>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="14">
         <f>B9+C8</f>
         <v/>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="14">
         <f>C9+D8</f>
         <v/>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="14">
         <f>D9+E8</f>
         <v/>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="14">
         <f>E9+F8</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="14">
         <f>F9+G8</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="14">
         <f>G9+H8</f>
         <v/>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="14">
         <f>H9+I8</f>
         <v/>
       </c>
-      <c r="J9" s="12">
+      <c r="J9" s="14">
         <f>I9+J8</f>
         <v/>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="14">
         <f>J9+K8</f>
         <v/>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="14">
         <f>K9+L8</f>
         <v/>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="14">
         <f>L9+M8</f>
         <v/>
       </c>
-      <c r="N9" s="14" t="n"/>
+      <c r="N9" s="16" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -2944,27 +3062,35 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>• Маржа 40% і OpEx 110 000 грн/міс — параметри (клітинка B5 і рядок 7), можна змінювати — модель перерахується.</t>
+          <t>• Маржа 40% (клітинка B5) і OpEx 380 000 грн/міс (рядок 7) — параметри, можна змінювати — модель перерахується.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>• Прогноз НЕ враховує повернення інвестиції (CapEx ~580–985 тис. грн) — окупність див. аркуш 7.</t>
+          <t>• Операційний беззбиток досягається з ~7-го місяця (травень 2027): валовий прибуток 392 тис. &gt; OpEx 380 тис.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>• Орієнтир: за цим сценарієм операційний беззбиток досягається з ~5-го місяця (березень 2027), річний операційний прибуток ~ +21 тис. грн (перший рік типово близький до нуля).</t>
+          <t>• Підсумок 1-го року — операційний мінус ≈ 0,5 млн грн (типово для роздробу). Саме тому в CapEx рекомендовано резерв ліквідності 3 міс. OpEx (~1,0–1,3 млн грн) і grace period по позиці.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>• Прогноз НЕ враховує повернення інвестиції (CapEx ~2,3–3,7 млн грн) — окупність див. аркуш 7.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A15:N15"/>
     <mergeCell ref="A11:N11"/>
     <mergeCell ref="A13:N13"/>
     <mergeCell ref="A14:N14"/>
@@ -2994,12 +3120,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Сценарії повернення інвестицій</t>
+          <t>Сценарії повернення інвестицій (ціни 2026)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>СЦЕНАРІЙ А. Позикове фінансування (ануїтет)</t>
         </is>
@@ -3012,9 +3138,13 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>600000</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
+        <v>2400000</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Покриває мінімальний CapEx</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3022,7 +3152,7 @@
           <t>Ставка, % річних</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="13" t="n">
         <v>0.12</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -3058,7 +3188,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>≈ 13 347 грн/міс.</t>
+          <t>≈ 53 400 грн/міс.</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3204,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>≈ 800 800 грн</t>
+          <t>≈ 3,20 млн грн</t>
         </is>
       </c>
     </row>
@@ -3090,21 +3220,21 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>≈ 200 800 грн за 5 років</t>
+          <t>≈ 0,80 млн грн за 5 років</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>Важливо: платіж ~13,3 тис. грн/міс. має покриватися операційним прибутком точки. За прогнозом 1-го року (аркуш 6) це навантаження критичне у перші 4–5 місяців — передбачити пільговий період (grace period) 6 місяців на тіло позики.</t>
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Важливо: платіж ~53 тис. грн/міс. має покриватися операційним прибутком точки. За прогнозом 1-го року (аркуш 6) у перші 6 місяців операційний прибуток від'ємний — обов'язково передбачити grace period 6–12 місяців на тіло позики та резерв ліквідності.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Графік погашення за роками (ануїтет 60 міс.)</t>
+          <t>Графік погашення за роками (ануїтет 60 міс., 2,4 млн грн під 12%)</t>
         </is>
       </c>
     </row>
@@ -3136,102 +3266,102 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Рік 1</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
-        <v>160160</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>93174</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>66986</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>506826</v>
+      <c r="B14" s="14" t="n">
+        <v>640640</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>372697</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>267944</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>2027303</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Рік 2</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>160160</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>104991</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>55169</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>401835</v>
+      <c r="B15" s="14" t="n">
+        <v>640640</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>419964</v>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>220676</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>1607340</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Рік 3</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>160160</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>118306</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>41854</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>283528</v>
+      <c r="B16" s="14" t="n">
+        <v>640640</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>473226</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>167414</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>1134114</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Рік 4</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>160160</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>133311</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>26849</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>150218</v>
+      <c r="B17" s="14" t="n">
+        <v>640640</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>533243</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>107397</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>600871</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Рік 5</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>160160</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>150218</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>9942</v>
-      </c>
-      <c r="E18" s="12" t="n">
+      <c r="B18" s="14" t="n">
+        <v>640640</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>600871</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>39769</v>
+      </c>
+      <c r="E18" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>СЦЕНАРІЙ Б. Частка від прибутку (profit-share)</t>
         </is>
@@ -3244,7 +3374,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>600000</v>
+        <v>2400000</v>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
     </row>
@@ -3254,7 +3384,7 @@
           <t>Частка інвестора у чистому прибутку</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="13" t="n">
         <v>0.3</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -3270,7 +3400,7 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>240000</v>
+        <v>960000</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
@@ -3290,7 +3420,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>≈ 72 000 грн/рік</t>
+          <t>≈ 288 000 грн/рік</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3430,7 @@
           <t>Простий строк повернення, років</t>
         </is>
       </c>
-      <c r="B25" s="17">
+      <c r="B25" s="19">
         <f>B21/B24</f>
         <v/>
       </c>
@@ -3311,14 +3441,14 @@
       </c>
     </row>
     <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>Висновок: profit-share 30% за прибутку 240 тис./рік повертає інвестицію ~8–10 років — повільно. Для привабливості або підвищити частку на перші роки (напр., 50% до повернення тіла), або комбінувати з позикою.</t>
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>Висновок: profit-share 30% за прибутку ~0,96 млн/рік повертає інвестицію ~8–10 років — повільно. Для привабливості або підвищити частку на перші роки (напр., 50% до повернення тіла), або комбінувати з позикою.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>СЦЕНАРІЙ В. Конвертація позики в частку нового ТОВ</t>
         </is>
@@ -3332,7 +3462,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Позика 600 тис. грн конвертується у 20–30% частки нового ТОВ при досягненні цільового EBIT (напр., 500 тис. грн/рік) або через 2–3 роки за оцінкою.</t>
+          <t>Позика 2,4 млн грн конвертується у 20–30% частки нового ТОВ при досягненні цільового EBIT (напр., 2 млн грн/рік) або через 2–3 роки за оцінкою.</t>
         </is>
       </c>
       <c r="C29" s="4" t="n"/>
@@ -3364,7 +3494,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>EBITDA 400 тис. грн/рік × 4 = оцінка 1,6 млн грн → позика 600 тис. ≈ 27% частки нового ТОВ (тільки офлайн-компанії).</t>
+          <t>EBITDA 1,6 млн грн/рік × 5 = оцінка 8,0 млн грн → позика 2,4 млн ≈ 30% частки нового ТОВ (тільки офлайн-компанії).</t>
         </is>
       </c>
       <c r="C31" s="4" t="n"/>
@@ -3434,7 +3564,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3610,7 +3740,7 @@
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>15000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="8">
@@ -3709,7 +3839,7 @@
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>10000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="11">
@@ -3742,7 +3872,7 @@
         </is>
       </c>
       <c r="G11" s="9" t="n">
-        <v>50000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="12">
@@ -3775,7 +3905,7 @@
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>10000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="13">
@@ -3841,7 +3971,7 @@
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>20000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="15">
@@ -3874,7 +4004,7 @@
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>25000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="16">
@@ -3907,7 +4037,7 @@
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>150000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="17">
@@ -3940,7 +4070,7 @@
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>50000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="18">
@@ -4006,7 +4136,7 @@
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>50000</v>
+        <v>175000</v>
       </c>
     </row>
     <row r="20">
@@ -4039,7 +4169,7 @@
         </is>
       </c>
       <c r="G20" s="9" t="n">
-        <v>300000</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="21">
@@ -4072,7 +4202,7 @@
         </is>
       </c>
       <c r="G21" s="9" t="n">
-        <v>20000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="22">
@@ -4105,7 +4235,7 @@
         </is>
       </c>
       <c r="G22" s="9" t="n">
-        <v>3000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="23">
@@ -4138,7 +4268,7 @@
         </is>
       </c>
       <c r="G23" s="9" t="n">
-        <v>40000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="24">
@@ -4171,7 +4301,7 @@
         </is>
       </c>
       <c r="G24" s="9" t="n">
-        <v>15000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="25">
@@ -4204,7 +4334,7 @@
         </is>
       </c>
       <c r="G25" s="9" t="n">
-        <v>3000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="26">
@@ -4237,7 +4367,7 @@
         </is>
       </c>
       <c r="G26" s="9" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="27">
@@ -4303,7 +4433,7 @@
         </is>
       </c>
       <c r="G28" s="9" t="n">
-        <v>30000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="29">
@@ -4340,36 +4470,36 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="n">
+      <c r="A30" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Запуск</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>УРОЧИСТЕ ВІДКРИТТЯ МАГАЗИНУ</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>15.11.2026</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>15.11.2026</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>ВІХА</t>
         </is>
       </c>
-      <c r="G30" s="19" t="n">
-        <v>10000</v>
+      <c r="G30" s="21" t="n">
+        <v>35000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove old-price comparison column and 2020 references
</commit_message>
<xml_diff>
--- a/Відкриття_фізичного_магазину.xlsx
+++ b/Відкриття_фізичного_магазину.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>План відкриття фізичного магазину footballshop.com.ua — повна версія (ціни 2026)</t>
+          <t>План відкриття фізичного магазину footballshop.com.ua — повна версія</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Діапазони витрат (мін/макс) у цінах 2026, беззбитковість, живі формули</t>
+          <t>Діапазони витрат (мін/макс), беззбитковість, живі формули</t>
         </is>
       </c>
     </row>
@@ -678,38 +678,30 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>• Суми актуалізовано до цін 2026 року (попередні оцінки 2020 р. збільшено у ~3–4 рази за рішенням власника: інфляція, девальвація, зростання оренди й зарплат).</t>
+          <t>• Усі суми — прогнозні; уточнити під конкретну локацію та орендні ставки.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>• Усі суми — прогнозні; уточнити під конкретну локацію та орендні ставки.</t>
+          <t>• Податкові ставки (станом на 2026) підтвердити з податковим консультантом — норми воєнного часу змінюються.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>• Податкові ставки (станом на 2026) підтвердити з податковим консультантом — норми воєнного часу змінюються.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>• КРИТИЧНО: з 06.01.2026 ПЗ 1С/BAS заборонено в Україні (рішення Держспецзв'язку, штрафи до 2% річного обороту). Bitrix і МойСклад — російського походження. Не використовувати.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2112,20 +2104,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Фінансова модель: магазин ~40–50 м², ціни 2026 (×3–4 від оцінок 2020), живі формули</t>
+          <t>Фінансова модель: магазин ~40–50 м² (діапазони мін–макс, живі формули)</t>
         </is>
       </c>
     </row>
@@ -2146,11 +2137,6 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Було (оцінка 2020), грн</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Коментар</t>
         </is>
@@ -2165,7 +2151,6 @@
       <c r="B4" s="8" t="n"/>
       <c r="C4" s="8" t="n"/>
       <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -2181,11 +2166,6 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>150–300 тис.</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
           <t>Залежить від стану приміщення</t>
         </is>
       </c>
@@ -2204,11 +2184,6 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>300–400 тис.</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
           <t>Глибина асортименту за брендами</t>
         </is>
       </c>
@@ -2227,11 +2202,6 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>50 тис.</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
           <t>Плюс банківський POS-термінал (від банку)</t>
         </is>
       </c>
@@ -2248,12 +2218,7 @@
       <c r="C8" s="9" t="n">
         <v>140000</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>25–40 тис.</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -2269,11 +2234,6 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>30–55 тис.</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
           <t>Юрист + реєстраційні платежі</t>
         </is>
       </c>
@@ -2292,11 +2252,6 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>60–90 тис.</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
           <t>Впровадження + інтеграція API</t>
         </is>
       </c>
@@ -2315,11 +2270,6 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
           <t>Повертається або зараховується</t>
         </is>
       </c>
@@ -2338,11 +2288,6 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>30–50 тис.</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
           <t>SMM + локальна реклама + відкриття</t>
         </is>
       </c>
@@ -2361,8 +2306,7 @@
         <f>SUM(C5:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Орієнтир: ~2,3–3,7 млн грн</t>
         </is>
@@ -2383,11 +2327,6 @@
         <v/>
       </c>
       <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Подушка на касові розриви першого року — НЕ входить у суму CapEx вище</t>
         </is>
@@ -2402,7 +2341,6 @@
       <c r="B15" s="8" t="n"/>
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2418,11 +2356,6 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>20–30 тис.</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
           <t>ТЦ або пішохідна вулиця</t>
         </is>
       </c>
@@ -2441,11 +2374,6 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>50 тис.</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
           <t>Менеджер + касир, по ~75–90 тис.</t>
         </is>
       </c>
@@ -2464,11 +2392,6 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>12–15 тис.</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
           <t>Нараховується на фонд оплати праці</t>
         </is>
       </c>
@@ -2485,12 +2408,7 @@
       <c r="C19" s="9" t="n">
         <v>25000</v>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>5–8 тис.</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2506,11 +2424,6 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>10–15 тис.</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
           <t>Постійне локальне просування</t>
         </is>
       </c>
@@ -2527,12 +2440,7 @@
       <c r="C21" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>5–10 тис.</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2548,11 +2456,6 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2–4 тис.</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
           <t>Checkbox + CRM + POS</t>
         </is>
       </c>
@@ -2571,8 +2474,7 @@
         <f>SUM(C16:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Орієнтир: ~325–449 тис. грн/міс.</t>
         </is>
@@ -2587,7 +2489,6 @@
       <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2601,8 +2502,7 @@
       <c r="C25" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Параметр — можна змінювати</t>
         </is>
@@ -2622,8 +2522,7 @@
         <f>C23/C26</f>
         <v/>
       </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>OpEx ÷ маржа ≈ 0,8–1,1 млн грн/міс.</t>
         </is>
@@ -2643,8 +2542,7 @@
         <f>C27*12</f>
         <v/>
       </c>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>≈ 9,8–13,5 млн грн/рік</t>
         </is>
@@ -2652,7 +2550,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2686,7 +2584,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Помісячний прогноз першого року роботи (P&amp;L), грн — листопад 2026 – жовтень 2027, ціни 2026</t>
+          <t>Помісячний прогноз першого року роботи (P&amp;L), грн — листопад 2026 – жовтень 2027</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3018,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Сценарії повернення інвестицій (ціни 2026)</t>
+          <t>Сценарії повернення інвестицій</t>
         </is>
       </c>
     </row>

</xml_diff>